<commit_message>
GBD: Excel de la 2FN completo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L4WdCDW8BpiQ7MhaaH9HRT
</commit_message>
<xml_diff>
--- a/0372-GBD-bases-de-datos/ejercicios/2026-10-17-nf1-ej3-normalizacion/2fn-ejercicio-3-2.xlsx
+++ b/0372-GBD-bases-de-datos/ejercicios/2026-10-17-nf1-ej3-normalizacion/2fn-ejercicio-3-2.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alumno" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curso" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matricula" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultado" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,15 +51,15 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -68,11 +69,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C00000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -117,16 +113,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -493,15 +486,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -515,19 +508,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Clave primaria (según el enunciado): codAlumno + codCurso</t>
+          <t>Clave primaria (según el enunciado): CodAlumno + CodCurso</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>codAlumno (PK)</t>
+          <t>CodAlumno (PK)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>codCurso (PK)</t>
+          <t>CodCurso (PK)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -552,7 +545,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>CreditosCurso</t>
+          <t>CréditosCurso</t>
         </is>
       </c>
     </row>
@@ -697,46 +690,73 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Pedro Ruiz</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>pedro@correo.com</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Programación I</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Luis Romero</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Celdas amarillas: completa con el resto de filas de tu enunciado (la captura de la VC03 solo enseña las primeras).</t>
-        </is>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>C30</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Laura Peña</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>laura@correo.com</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Redes</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Carlos Rubio</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -750,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -769,7 +789,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>La clave es compuesta (codAlumno, codCurso) y hay dependencias parciales.</t>
+          <t>La clave es compuesta (CodAlumno, CodCurso) y hay dependencias parciales.</t>
         </is>
       </c>
     </row>
@@ -801,17 +821,17 @@
           <t>NombreAlumno</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Solo el alumno: A01 siempre es Marta López</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>codAlumno</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
+          <t>CodAlumno</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Parcial ❌</t>
         </is>
@@ -823,17 +843,17 @@
           <t>EmailAlumno</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Solo el alumno: A01 siempre es marta@correo.com</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>codAlumno</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+          <t>CodAlumno</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Parcial ❌</t>
         </is>
@@ -845,17 +865,17 @@
           <t>NombreCurso</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Solo el curso: C10 siempre es Bases de Datos</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>codCurso</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
+          <t>CodCurso</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Parcial ❌</t>
         </is>
@@ -867,17 +887,17 @@
           <t>ProfesorCurso</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Solo el curso: C10 siempre es Ana Martínez</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>codCurso</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
+          <t>CodCurso</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Parcial ❌</t>
         </is>
@@ -886,43 +906,57 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CreditosCurso</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
+          <t>CréditosCurso</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Solo el curso: C10 siempre tiene 6 créditos</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>codCurso</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
+          <t>CodCurso</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Parcial ❌</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Ninguna columna depende de los dos campos de la clave a la vez.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Pista visual: «Marta López» y su email se repiten en cada curso; «Bases de Datos / Ana Martínez / 6» se repite en cada alumno del C10.</t>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Consecuencia (redundancia): Marta López y su email se repiten 3 veces; Pedro Ruiz 2 veces;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Solución: separar lo que depende de codAlumno (tabla Alumno), lo que depende de codCurso (tabla Curso) y dejar la clave completa en Matricula.</t>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>«Bases de Datos / Ana Martínez / 6», «Programación I / Luis Romero / 8» y «Redes / Carlos Rubio / 5» se repiten 2 veces cada uno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Proceso: lo que depende solo de CodAlumno va a la tabla Alumno; lo que depende solo de CodCurso va a la tabla Curso;</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>la tabla original se queda solo con la clave completa (Matricula), cuyos campos pasan a ser PK y FK.</t>
         </is>
       </c>
     </row>
@@ -937,12 +971,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1004,24 +1038,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Celdas amarillas: completa con el resto de filas de tu enunciado (la captura de la VC03 solo enseña las primeras).</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Laura Peña</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>laura@correo.com</t>
         </is>
       </c>
     </row>
@@ -1036,12 +1065,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -1132,25 +1161,6 @@
       </c>
       <c r="D6" s="4" t="n">
         <v>5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Celdas amarillas: completa con el resto de filas de tu enunciado (la captura de la VC03 solo enseña las primeras).</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1164,7 +1174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1181,7 +1191,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Una fila por cada fila de la tabla original. El nombre «Matricula» no lo da el enunciado (también vale «AlumnoCurso»).</t>
+          <t>Es la tabla original tras la normalización: solo queda la clave. El nombre «Matricula» no lo da el enunciado (también vale «AlumnoCurso»).</t>
         </is>
       </c>
     </row>
@@ -1246,25 +1256,183 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Celdas amarillas: completa con el resto de filas de tu enunciado (la captura de la VC03 solo enseña las primeras).</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>C30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Diseño resultante en 2FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Tabla</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Otros atributos</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Qué guarda</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Alumno</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>codAlumno</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>nombreAlumno, emailAlumno</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Datos de cada alumno. Cada alumno aparece una sola vez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>codCurso</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>nombreCurso, profesorCurso, creditosCurso</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Datos de cada curso. Cada curso aparece una sola vez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Matricula</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>codAlumno + codCurso</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>codAlumno → Alumno; codCurso → Curso</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Qué alumno está en qué curso. Es la tabla original tras la normalización.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Por qué ya está en 2FN:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Alumno y Curso tienen clave simple, así que no puede haber dependencias parciales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Matricula tiene clave compuesta, pero no tiene más atributos que la clave.</t>
         </is>
       </c>
     </row>

</xml_diff>